<commit_message>
Regenerate showcase downloads against the unified API
</commit_message>
<xml_diff>
--- a/Website/static/downloads/showcase/workflows/excel-asset-depreciation/example.xlsx
+++ b/Website/static/downloads/showcase/workflows/excel-asset-depreciation/example.xlsx
@@ -1,13 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:bookViews xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:bookViews>
     <x:workbookView/>
   </x:bookViews>
-  <sheets>
-    <sheet name="Assets" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="1" r:id="R83d44ad3ac454fa8"/>
+  </x:sheets>
+  <x:definedNames>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="0">'Assets'!$4:$4</x:definedName>
+  </x:definedNames>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -65,56 +68,41 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
-      <x:name val="Calibri"/>
+      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:sz val="22"/>
-      <x:name val="Calibri"/>
+      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="22"/>
-      <x:name val="Calibri"/>
+      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="22"/>
       <x:color rgb="FF17365D"/>
-      <x:name val="Calibri"/>
+      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="22"/>
-      <x:color rgb="FF17365D"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:name val="Carlito"/>
+      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
+      <x:name val="Aptos"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
+      <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
   <x:fills count="3">
@@ -137,20 +125,33 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
     <x:xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -175,8 +176,294 @@
 </x:table>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="OfficeIMO Modern">
+  <a:themeElements>
+    <a:clrScheme name="Modern">
+      <a:dk1>
+        <a:srgbClr val="1B2433"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="5B6575"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="F6F8FB"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="3F64D7"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="DC7536"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="058E80"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="A52758"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="3F2F6B"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="255319"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="3F64D7"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="A52758"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Modern">
+      <a:majorFont>
+        <a:latin typeface="Aptos"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <x:sheetPr xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
   <dimension ref="A1:F16"/>
   <x:sheetFormatPr xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" defaultRowHeight="15"/>
   <cols>
@@ -189,14 +476,9 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
     </row>
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="7" t="s">
@@ -220,13 +502,13 @@
       <c r="A4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="15" t="s">
         <v>5</v>
       </c>
       <c r="E4" s="12" t="s">
@@ -240,20 +522,20 @@
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>7200</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="9" t="n">
         <v>600</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="9" t="n">
         <x:f xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ca="0">(B5-C5)/D5</x:f>
         <v>2200</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="9" t="n">
         <x:f xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ca="0">B5-E5</x:f>
         <v>5000</v>
       </c>
@@ -262,20 +544,20 @@
       <c r="A6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>3600</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="9" t="n">
         <v>300</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="9" t="n">
         <x:f xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ca="0">(B6-C6)/D6</x:f>
         <v>825</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="9" t="n">
         <x:f xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ca="0">B6-E6</x:f>
         <v>2775</v>
       </c>
@@ -284,20 +566,20 @@
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>9200</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="9" t="n">
         <v>800</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="9" t="n">
         <x:f xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ca="0">(B7-C7)/D7</x:f>
         <v>1680</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="9" t="n">
         <x:f xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ca="0">B7-E7</x:f>
         <v>7520</v>
       </c>
@@ -306,20 +588,20 @@
       <c r="A8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>4800</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="9" t="n">
         <v>400</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="9" t="n">
         <x:f xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ca="0">(B8-C8)/D8</x:f>
         <v>1100</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="9" t="n">
         <x:f xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ca="0">B8-E8</x:f>
         <v>3700</v>
       </c>
@@ -339,7 +621,7 @@
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="6" t="n">
         <x:f xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ca="0">SUM(E5:E8)</x:f>
         <v>5805</v>
       </c>
@@ -410,6 +692,7 @@
       <x:formula2>50</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
+  <x:pageSetup xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" fitToWidth="1" fitToHeight="0" orientation="landscape"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>